<commit_message>
Update: Fixed Packing PO Start Date/time and End Date/Time
</commit_message>
<xml_diff>
--- a/APPT/data/input/equipment_master.xlsx
+++ b/APPT/data/input/equipment_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pratyush\Desktop\ARX\ARX-SFA Projects\P&amp;G\PG-AutoProdTool\APPT\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C9760D4-E865-4876-BBA5-02800513E84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAD637CD-F4D5-40C2-9602-3BE086591083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="62">
   <si>
     <t>TK#_1_#</t>
   </si>
@@ -138,9 +138,6 @@
     <t>TK#_9_#</t>
   </si>
   <si>
-    <t>equipment_id</t>
-  </si>
-  <si>
     <t>equip_type</t>
   </si>
   <si>
@@ -199,6 +196,21 @@
   </si>
   <si>
     <t>resource group</t>
+  </si>
+  <si>
+    <t>12T</t>
+  </si>
+  <si>
+    <t>FMT</t>
+  </si>
+  <si>
+    <t>Mix</t>
+  </si>
+  <si>
+    <t>6T</t>
+  </si>
+  <si>
+    <t>MMT</t>
   </si>
 </sst>
 </file>
@@ -241,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -264,11 +276,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -280,6 +305,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,809 +593,750 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultColWidth="25.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.90625" customWidth="1"/>
-    <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" customWidth="1"/>
-    <col min="4" max="4" width="20.453125" customWidth="1"/>
-    <col min="5" max="5" width="20.54296875" customWidth="1"/>
+    <col min="2" max="2" width="13.6328125" customWidth="1"/>
+    <col min="3" max="3" width="20.453125" customWidth="1"/>
+    <col min="4" max="4" width="20.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
-        <v>11</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4">
-        <v>14</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4">
-        <v>16</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4">
-        <v>17</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4">
-        <v>18</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4">
-        <v>19</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="B12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4">
-        <v>2</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4">
-        <v>20</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B14" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4">
-        <v>21</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="4">
-        <v>22</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4">
-        <v>23</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="B17" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="4">
-        <v>24</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="4">
-        <v>25</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B19" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="4">
-        <v>26</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="4">
-        <v>27</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="4">
-        <v>28</v>
-      </c>
-      <c r="C22" s="4" t="s">
+      <c r="B22" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="4">
-        <v>3</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="B23" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="4">
-        <v>37</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>41</v>
+      <c r="B24" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="4">
-        <v>38</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>41</v>
+      <c r="B25" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="4">
-        <v>4</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="4">
-        <v>5</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="B27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F27" s="2"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="4">
-        <v>51</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>41</v>
+      <c r="B28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F28" s="2"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="4">
-        <v>52</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>41</v>
+      <c r="B29" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="4">
-        <v>53</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>41</v>
+      <c r="B30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="4">
-        <v>56</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>41</v>
+      <c r="B31" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F31" s="2"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="4">
-        <v>57</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>41</v>
+      <c r="B32" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="4">
-        <v>58</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>41</v>
+      <c r="B33" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="4">
-        <v>59</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>41</v>
+      <c r="B34" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="4">
-        <v>6</v>
-      </c>
-      <c r="C35" s="4" t="s">
+      <c r="B35" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="4">
-        <v>7</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="B36" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F36" s="2"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="4">
-        <v>8</v>
-      </c>
-      <c r="C37" s="4" t="s">
+      <c r="B37" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="4">
-        <v>9</v>
-      </c>
-      <c r="C38" s="4" t="s">
+      <c r="B38" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F38" s="2"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D39" s="2" t="s">
+      <c r="D43" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E39" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F40" s="2"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F42" s="2"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F43" s="2"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F44" s="2"/>
+      <c r="D44" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="7"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="3"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="3"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>